<commit_message>
let F3 show the pathways only HR bothered to move
</commit_message>
<xml_diff>
--- a/04_Figures/F4/c_data/F4.xlsx
+++ b/04_Figures/F4/c_data/F4.xlsx
@@ -170,7 +170,7 @@
     <t>label</t>
   </si>
   <si>
-    <t>Set name as printed in the figure; * marks calls of opposite sign within the window.</t>
+    <t>Set name as printed in the figure; * marks calls of opposite sign within the window; † a training or acute set whose interaction also reaches FDR &lt; 0.05.</t>
   </si>
   <si>
     <t>nes</t>
@@ -659,7 +659,7 @@
     <t>Reactome|REACTOME_ASPARAGINE_N_LINKED_GLYCOSYLATION</t>
   </si>
   <si>
-    <t>Asparagine n linked glycosylation</t>
+    <t>Asparagine N linked glycosylation</t>
   </si>
   <si>
     <t>Reactome|REACTOME_CELLULAR_SENESCENCE</t>

</xml_diff>

<commit_message>
set F3 counts beside the pathways so the gap speaks for itself
</commit_message>
<xml_diff>
--- a/04_Figures/F4/c_data/F4.xlsx
+++ b/04_Figures/F4/c_data/F4.xlsx
@@ -521,7 +521,7 @@
     <t>Reactome|REACTOME_AEROBIC_RESPIRATION_AND_RESPIRATORY_ELECTRON_TRANSPORT</t>
   </si>
   <si>
-    <t>Aerobic respiration and respiratory electron tran...</t>
+    <t>Aerobic respiration and respiratory electron transport</t>
   </si>
   <si>
     <t>GOBP|GOBP_TRICARBOXYLIC_ACID_CYCLE</t>
@@ -629,13 +629,13 @@
     <t>GOBP|GOBP_REGULATION_OF_ESTABLISHMENT_OF_PROTEIN_LOCALIZATION_TO_MITOCHONDRION</t>
   </si>
   <si>
-    <t>Regulation of establishment of protein localizati...</t>
+    <t>Regulation of establishment of protein localization to mitoch...</t>
   </si>
   <si>
     <t>GOBP|GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_CELL_PERIPHERY</t>
   </si>
   <si>
-    <t>Positive regulation of protein localization to ce...</t>
+    <t>Positive regulation of protein localization to cell periphery</t>
   </si>
   <si>
     <t>Reactome|REACTOME_EPIGENETIC_REGULATION_OF_GENE_EXPRESSION</t>
@@ -671,7 +671,7 @@
     <t>GOBP|GOBP_ENDOPLASMIC_RETICULUM_TO_GOLGI_VESICLE_MEDIATED_TRANSPORT</t>
   </si>
   <si>
-    <t>Endoplasmic reticulum to Golgi vesicle mediated t...</t>
+    <t>Endoplasmic reticulum to Golgi vesicle mediated transport</t>
   </si>
   <si>
     <t>GOBP|GOBP_STRIATED_MUSCLE_ADAPTATION</t>
@@ -689,7 +689,7 @@
     <t>GOBP|GOBP_NEGATIVE_REGULATION_OF_SYNCYTIUM_FORMATION_BY_PLASMA_MEMBRANE_FUSION</t>
   </si>
   <si>
-    <t>Negative regulation of syncytium formation by pla...</t>
+    <t>Negative regulation of syncytium formation by plasma membrane...</t>
   </si>
   <si>
     <t>Reactome|REACTOME_RHO_GTPASES_ACTIVATE_PKNS</t>

</xml_diff>